<commit_message>
Add optional fields to spreadsheet import examples
</commit_message>
<xml_diff>
--- a/product-options-manager/public/examples/product-options-example.xlsx
+++ b/product-options-manager/public/examples/product-options-example.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size and Quantity" sheetId="1" r:id="R9a2084e5850b4074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size Color and Quantity" sheetId="2" r:id="R60b7b99d20f84a4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Product Rates" sheetId="3" r:id="Rb79049df54a140ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size and Quantity" sheetId="1" r:id="Rddbff39e2bca4875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size Color and Quantity" sheetId="2" r:id="R976fef83baa8479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shared Product Rates" sheetId="3" r:id="Rd945e917580f4742"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size GSM and Quantity" sheetId="4" r:id="Rc0ef2f2273094097"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,6 +47,12 @@
       <x:name val="Arial"/>
     </x:font>
     <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF202223"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF4A4F55"/>
       <x:name val="Arial"/>
@@ -57,7 +64,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -67,6 +74,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF254438"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEBE2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F8FA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -82,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -96,8 +113,20 @@
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -300,11 +329,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
@@ -479,43 +508,210 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="10" t="str">
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="10" t="str">
+        <x:v>EXTRA FIELDS</x:v>
+      </x:c>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="1"/>
+      <x:c r="E12" s="1"/>
+      <x:c r="F12" s="1"/>
+      <x:c r="G12" s="1"/>
+      <x:c r="H12" s="1"/>
+      <x:c r="I12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="11" t="str">
+        <x:v>Label</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>Values</x:v>
+      </x:c>
+      <x:c r="F13" s="1"/>
+      <x:c r="G13" s="1"/>
+      <x:c r="H13" s="1"/>
+      <x:c r="I13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>GSM</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>220 gsm|300 gsm|400 gsm</x:v>
+      </x:c>
+      <x:c r="F14" s="14"/>
+      <x:c r="G14" s="14"/>
+      <x:c r="H14" s="14"/>
+      <x:c r="I14" s="14"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>Logo Upload</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>upload</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str"/>
+      <x:c r="F15" s="14"/>
+      <x:c r="G15" s="14"/>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="14"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>Enter Pincode</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str"/>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Printing</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>No Printing|Front Only|Both Sides</x:v>
+      </x:c>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Order Notes</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str"/>
+      <x:c r="F18" s="14"/>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>Delivery Date</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str"/>
+      <x:c r="F19" s="14"/>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="14"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="16" t="str">
         <x:v>HOW TO USE</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="9" t="str">
+    <x:row r="23">
+      <x:c r="A23" s="15" t="str">
+        <x:v>EXTRA FIELDS: Enabled Yes creates a field; No skips it. Required Yes makes entry mandatory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="15" t="str">
+        <x:v>Types: text, number, date, upload, radio, dropdown. Separate choices with | in Values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="15" t="str">
+        <x:v>Extra fields do not affect prices. For priced GSM use the Size GSM and Quantity tab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="15" t="str">
         <x:v>Replace the group name in row 1 and every sample product URL above the table.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="9" t="str">
+    <x:row r="27">
+      <x:c r="A27" s="15" t="str">
         <x:v>Keep one product URL per row. All listed products share this table’s options and rates.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="9" t="str">
+    <x:row r="28">
+      <x:c r="A28" s="15" t="str">
         <x:v>Edit the option values and quantity headers. Add new combinations directly below the sample rows.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="9" t="str">
+    <x:row r="29">
+      <x:c r="A29" s="15" t="str">
         <x:v>Enter per-piece rates in the table. The importer calculates quantity × rate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="9" t="str">
+    <x:row r="30">
+      <x:c r="A30" s="15" t="str">
         <x:v>Example: quantity 10 at rate 180 becomes a total price of Rs. 1,800.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="9" t="str">
+    <x:row r="31">
+      <x:c r="A31" s="15" t="str">
         <x:v>Keep only the example tabs you need. Duplicate a tab for another product or group.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="9" t="str">
+    <x:row r="32">
+      <x:c r="A32" s="15" t="str">
         <x:v>Save as .xlsx, upload in Import spreadsheet, review the preview, then import.</x:v>
       </x:c>
     </x:row>
@@ -528,11 +724,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
@@ -788,43 +984,218 @@
         <x:v>130</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="10" t="str">
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="10" t="str">
+        <x:v>EXTRA FIELDS</x:v>
+      </x:c>
+      <x:c r="B14" s="1"/>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="1"/>
+      <x:c r="E14" s="1"/>
+      <x:c r="F14" s="1"/>
+      <x:c r="G14" s="1"/>
+      <x:c r="H14" s="1"/>
+      <x:c r="I14" s="1"/>
+      <x:c r="J14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="11" t="str">
+        <x:v>Label</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="str">
+        <x:v>Values</x:v>
+      </x:c>
+      <x:c r="F15" s="1"/>
+      <x:c r="G15" s="1"/>
+      <x:c r="H15" s="1"/>
+      <x:c r="I15" s="1"/>
+      <x:c r="J15" s="1"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>GSM</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>220 gsm|300 gsm|400 gsm</x:v>
+      </x:c>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+      <x:c r="J16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Logo Upload</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>upload</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str"/>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+      <x:c r="J17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Enter Pincode</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str"/>
+      <x:c r="F18" s="14"/>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+      <x:c r="J18" s="14"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>Printing</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str">
+        <x:v>No Printing|Front Only|Both Sides</x:v>
+      </x:c>
+      <x:c r="F19" s="14"/>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="14"/>
+      <x:c r="J19" s="14"/>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="12" t="str">
+        <x:v>Order Notes</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E20" s="13" t="str"/>
+      <x:c r="F20" s="14"/>
+      <x:c r="G20" s="14"/>
+      <x:c r="H20" s="14"/>
+      <x:c r="I20" s="14"/>
+      <x:c r="J20" s="14"/>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="12" t="str">
+        <x:v>Delivery Date</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E21" s="13" t="str"/>
+      <x:c r="F21" s="14"/>
+      <x:c r="G21" s="14"/>
+      <x:c r="H21" s="14"/>
+      <x:c r="I21" s="14"/>
+      <x:c r="J21" s="14"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="16" t="str">
         <x:v>HOW TO USE</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="9" t="str">
+    <x:row r="25">
+      <x:c r="A25" s="15" t="str">
+        <x:v>EXTRA FIELDS: Enabled Yes creates a field; No skips it. Required Yes makes entry mandatory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="15" t="str">
+        <x:v>Types: text, number, date, upload, radio, dropdown. Separate choices with | in Values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="15" t="str">
+        <x:v>Extra fields do not affect prices. For priced GSM use the Size GSM and Quantity tab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="15" t="str">
         <x:v>Replace the group name in row 1 and every sample product URL above the table.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="9" t="str">
+    <x:row r="29">
+      <x:c r="A29" s="15" t="str">
         <x:v>Keep one product URL per row. All listed products share this table’s options and rates.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="9" t="str">
+    <x:row r="30">
+      <x:c r="A30" s="15" t="str">
         <x:v>Edit the option values and quantity headers. Add new combinations directly below the sample rows.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="9" t="str">
+    <x:row r="31">
+      <x:c r="A31" s="15" t="str">
         <x:v>Enter per-piece rates in the table. The importer calculates quantity × rate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="9" t="str">
+    <x:row r="32">
+      <x:c r="A32" s="15" t="str">
         <x:v>Example: quantity 10 at rate 180 becomes a total price of Rs. 1,800.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="9" t="str">
+    <x:row r="33">
+      <x:c r="A33" s="15" t="str">
         <x:v>Keep only the example tabs you need. Duplicate a tab for another product or group.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="9" t="str">
+    <x:row r="34">
+      <x:c r="A34" s="15" t="str">
         <x:v>Save as .xlsx, upload in Import spreadsheet, review the preview, then import.</x:v>
       </x:c>
     </x:row>
@@ -837,11 +1208,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
@@ -991,43 +1362,630 @@
         <x:v>90</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="10" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="10" t="str">
+        <x:v>EXTRA FIELDS</x:v>
+      </x:c>
+      <x:c r="B11" s="1"/>
+      <x:c r="C11" s="1"/>
+      <x:c r="D11" s="1"/>
+      <x:c r="E11" s="1"/>
+      <x:c r="F11" s="1"/>
+      <x:c r="G11" s="1"/>
+      <x:c r="H11" s="1"/>
+      <x:c r="I11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="11" t="str">
+        <x:v>Label</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="str">
+        <x:v>Values</x:v>
+      </x:c>
+      <x:c r="F12" s="1"/>
+      <x:c r="G12" s="1"/>
+      <x:c r="H12" s="1"/>
+      <x:c r="I12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>GSM</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="str">
+        <x:v>220 gsm|300 gsm|400 gsm</x:v>
+      </x:c>
+      <x:c r="F13" s="14"/>
+      <x:c r="G13" s="14"/>
+      <x:c r="H13" s="14"/>
+      <x:c r="I13" s="14"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>Logo Upload</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>upload</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str"/>
+      <x:c r="F14" s="14"/>
+      <x:c r="G14" s="14"/>
+      <x:c r="H14" s="14"/>
+      <x:c r="I14" s="14"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>Enter Pincode</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str"/>
+      <x:c r="F15" s="14"/>
+      <x:c r="G15" s="14"/>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="14"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>Printing</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str">
+        <x:v>No Printing|Front Only|Both Sides</x:v>
+      </x:c>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Order Notes</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str"/>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Delivery Date</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str"/>
+      <x:c r="F18" s="14"/>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="16" t="str">
         <x:v>HOW TO USE</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="9" t="str">
+    <x:row r="22">
+      <x:c r="A22" s="15" t="str">
+        <x:v>EXTRA FIELDS: Enabled Yes creates a field; No skips it. Required Yes makes entry mandatory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="15" t="str">
+        <x:v>Types: text, number, date, upload, radio, dropdown. Separate choices with | in Values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="15" t="str">
+        <x:v>Extra fields do not affect prices. For priced GSM use the Size GSM and Quantity tab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="15" t="str">
         <x:v>Replace the group name in row 1 and every sample product URL above the table.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="9" t="str">
+    <x:row r="26">
+      <x:c r="A26" s="15" t="str">
         <x:v>Keep one product URL per row. All listed products share this table’s options and rates.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="9" t="str">
+    <x:row r="27">
+      <x:c r="A27" s="15" t="str">
         <x:v>Edit the option values and quantity headers. Add new combinations directly below the sample rows.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="9" t="str">
+    <x:row r="28">
+      <x:c r="A28" s="15" t="str">
         <x:v>Enter per-piece rates in the table. The importer calculates quantity × rate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="9" t="str">
+    <x:row r="29">
+      <x:c r="A29" s="15" t="str">
         <x:v>Example: quantity 10 at rate 180 becomes a total price of Rs. 1,800.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="9" t="str">
+    <x:row r="30">
+      <x:c r="A30" s="15" t="str">
         <x:v>Keep only the example tabs you need. Duplicate a tab for another product or group.</x:v>
       </x:c>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="15" t="str">
+        <x:v>Save as .xlsx, upload in Import spreadsheet, review the preview, then import.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>GSM priced bag options</x:v>
+      </x:c>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>https://your-store.myshopify.com/products/replace-with-gsm-bag-handle</x:v>
+      </x:c>
+      <x:c r="B2" s="1"/>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1"/>
+      <x:c r="J2" s="1"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="1"/>
+      <x:c r="B4" s="1"/>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+      <x:c r="E4" s="1"/>
+      <x:c r="F4" s="1"/>
+      <x:c r="G4" s="1"/>
+      <x:c r="H4" s="1"/>
+      <x:c r="I4" s="1"/>
+      <x:c r="J4" s="1"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="1"/>
+      <x:c r="B5" s="1"/>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+      <x:c r="E5" s="1"/>
+      <x:c r="F5" s="1"/>
+      <x:c r="G5" s="1"/>
+      <x:c r="H5" s="1"/>
+      <x:c r="I5" s="1"/>
+      <x:c r="J5" s="1"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="1"/>
+      <x:c r="B6" s="1"/>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="1"/>
+      <x:c r="G6" s="1"/>
+      <x:c r="H6" s="1"/>
+      <x:c r="I6" s="1"/>
+      <x:c r="J6" s="1"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="1"/>
+      <x:c r="B7" s="1"/>
+      <x:c r="C7" s="1"/>
+      <x:c r="D7" s="1"/>
+      <x:c r="E7" s="1"/>
+      <x:c r="F7" s="1"/>
+      <x:c r="G7" s="1"/>
+      <x:c r="H7" s="1"/>
+      <x:c r="I7" s="1"/>
+      <x:c r="J7" s="1"/>
+    </x:row>
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>Sl No</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>Size</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>GSM</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="I8" s="6" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="str">
+        <x:v>Small</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>220 gsm</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="H9" s="8" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="I9" s="8" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J9" s="8" t="n">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="str">
+        <x:v>Small</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="str">
+        <x:v>400 gsm</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="E10" s="8" t="n">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="G10" s="8" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="H10" s="8" t="n">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="I10" s="8" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="J10" s="8" t="n">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="10" t="str">
+        <x:v>EXTRA FIELDS</x:v>
+      </x:c>
+      <x:c r="B12" s="1"/>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="1"/>
+      <x:c r="E12" s="1"/>
+      <x:c r="F12" s="1"/>
+      <x:c r="G12" s="1"/>
+      <x:c r="H12" s="1"/>
+      <x:c r="I12" s="1"/>
+      <x:c r="J12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="11" t="str">
+        <x:v>Label</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>Values</x:v>
+      </x:c>
+      <x:c r="F13" s="1"/>
+      <x:c r="G13" s="1"/>
+      <x:c r="H13" s="1"/>
+      <x:c r="I13" s="1"/>
+      <x:c r="J13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>GSM</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="str">
+        <x:v>220 gsm|300 gsm|400 gsm</x:v>
+      </x:c>
+      <x:c r="F14" s="14"/>
+      <x:c r="G14" s="14"/>
+      <x:c r="H14" s="14"/>
+      <x:c r="I14" s="14"/>
+      <x:c r="J14" s="14"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>Logo Upload</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>upload</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str"/>
+      <x:c r="F15" s="14"/>
+      <x:c r="G15" s="14"/>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="14"/>
+      <x:c r="J15" s="14"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>Enter Pincode</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>number</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E16" s="13" t="str"/>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+      <x:c r="J16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Printing</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>dropdown</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E17" s="13" t="str">
+        <x:v>No Printing|Front Only|Both Sides</x:v>
+      </x:c>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+      <x:c r="J17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Order Notes</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E18" s="13" t="str"/>
+      <x:c r="F18" s="14"/>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+      <x:c r="J18" s="14"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>Delivery Date</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E19" s="13" t="str"/>
+      <x:c r="F19" s="14"/>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="14"/>
+      <x:c r="J19" s="14"/>
+    </x:row>
     <x:row r="22">
-      <x:c r="A22" s="9" t="str">
+      <x:c r="A22" s="16" t="str">
+        <x:v>HOW TO USE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="15" t="str">
+        <x:v>EXTRA FIELDS: Enabled Yes creates a field; No skips it. Required Yes makes entry mandatory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="15" t="str">
+        <x:v>Types: text, number, date, upload, radio, dropdown. Separate choices with | in Values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="15" t="str">
+        <x:v>Extra fields do not affect prices. For priced GSM use the Size GSM and Quantity tab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="15" t="str">
+        <x:v>Replace the group name in row 1 and every sample product URL above the table.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="15" t="str">
+        <x:v>Keep one product URL per row. All listed products share this table’s options and rates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="15" t="str">
+        <x:v>Edit the option values and quantity headers. Add new combinations directly below the sample rows.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="15" t="str">
+        <x:v>Enter per-piece rates in the table. The importer calculates quantity × rate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="15" t="str">
+        <x:v>Example: quantity 10 at rate 180 becomes a total price of Rs. 1,800.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="15" t="str">
+        <x:v>Keep only the example tabs you need. Duplicate a tab for another product or group.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="15" t="str">
         <x:v>Save as .xlsx, upload in Import spreadsheet, review the preview, then import.</x:v>
       </x:c>
     </x:row>

</xml_diff>